<commit_message>
Correction LOG0009 T3 et reservation directe
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/ReservationsHH/SAISIE_ReservationsHorsHostaway.xlsx
+++ b/01_SOURCES_BRUTES/ReservationsHH/SAISIE_ReservationsHorsHostaway.xlsx
@@ -32,7 +32,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="5">
     <font>
       <name val="Calibri"/>
@@ -146,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -182,6 +184,7 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -753,6 +756,11 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>RESHH-2026-05-001</t>
+        </is>
+      </c>
       <c r="B2">
         <f>IF(A2="","",A2&amp;"|"&amp;D2&amp;"|"&amp;F2&amp;"|"&amp;G2&amp;"|"&amp;TEXT(I2,"YYYYMMDD")&amp;"|"&amp;TEXT(L2,"0.00"))</f>
         <v/>
@@ -761,10 +769,45 @@
         <f>IF(I2="","",TEXT(I2,"YYYY-MM"))</f>
         <v/>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CANAL_004</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>DIRECT_HA_PAYANT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PROP_0003</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>LOG_0009</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>60559486</v>
+      </c>
+      <c r="I2" s="15" t="n">
+        <v>46167</v>
+      </c>
+      <c r="J2" s="15" t="n">
+        <v>46222</v>
+      </c>
       <c r="K2">
         <f>IF(OR(I2="",J2=""),"",J2-I2)</f>
         <v/>
       </c>
+      <c r="L2" t="n">
+        <v>2343.48</v>
+      </c>
+      <c r="M2" t="n">
+        <v>55</v>
+      </c>
       <c r="N2">
         <f>IF(F2="","",IFERROR(VLOOKUP(F2,lst_PropTauxLookup,2,0),""))</f>
         <v/>
@@ -781,6 +824,16 @@
         <f>IF(L2="","",L2-IF(M2="",0,M2)-IF(Q2="",0,Q2)-IF(T2="",0,T2))</f>
         <v/>
       </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>HC</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>NON</t>
+        </is>
+      </c>
       <c r="Y2">
         <f>IF(W2="IC","OUI",IF(W2="HC","OUI",IF(W2="HR","NON","A_CONTROLER")))</f>
         <v/>
@@ -788,6 +841,21 @@
       <c r="Z2">
         <f>IF(W2="IC","OUI",IF(W2="HC","NON",IF(W2="HR","NON","A_CONTROLER")))</f>
         <v/>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>VALIDE</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>Reservation directe Hostaway 60559486 integree (decision humaine 2026-06-15). Menage standard T3 deduit pour assiette commission.</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -20404,7 +20472,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -20426,7 +20493,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -20448,7 +20514,6 @@
           <t>ATTENTION si &gt; 0</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -20470,7 +20535,6 @@
           <t>INFO</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -20492,7 +20556,6 @@
           <t>ATTENTION si &gt; 0</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
Supprime doublons sources verite et securise imports
</commit_message>
<xml_diff>
--- a/01_SOURCES_BRUTES/ReservationsHH/SAISIE_ReservationsHorsHostaway.xlsx
+++ b/01_SOURCES_BRUTES/ReservationsHH/SAISIE_ReservationsHorsHostaway.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="SAISIE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="REF_LOCALE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CONTROLES_SAISIE" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SAISIE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LOCALE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CONTROLES_SAISIE" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="lst_Canaux">'REF_LOCALE'!$A$2:$A$6</definedName>
@@ -20903,7 +20903,7 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>5. taux_commission : pre-rempli via VLOOKUP depuis REF_Proprietaires (col N).</t>
+          <t>5. taux_commission : resolu en aval depuis REF_Taux_Commission ; ne pas saisir de taux non date.</t>
         </is>
       </c>
     </row>

</xml_diff>